<commit_message>
finalizacion de las pruebas para las funciones faltantes: incluyendo para read_write_multiple_registers y read_fifo_queue, se deben verificar el maximo de bytes despues en la libreria ya que en ciertos casos puede ser menor
</commit_message>
<xml_diff>
--- a/modbus.xlsx
+++ b/modbus.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\windows\projects\rust\firerust\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6B7D9A-E605-4385-9341-A4EB4C479602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF1632D5-EEB3-49F5-BCEC-6E85FABDB37C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -215,9 +215,6 @@
     <t>write_file_record</t>
   </si>
   <si>
-    <t>mask_write_record</t>
-  </si>
-  <si>
     <t>01 17 00 00 00 02 00 0A 00 02 04 00 01 00 02 E2 63</t>
   </si>
   <si>
@@ -270,6 +267,9 @@
   </si>
   <si>
     <t>01 0C 00 25</t>
+  </si>
+  <si>
+    <t>mask_write_register</t>
   </si>
 </sst>
 </file>
@@ -374,16 +374,16 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -645,56 +645,56 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:28" ht="30" customHeight="1">
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="16"/>
-      <c r="F2" s="13" t="s">
+      <c r="E2" s="13"/>
+      <c r="F2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="14" t="s">
         <v>5</v>
       </c>
       <c r="I2" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="14" t="s">
         <v>7</v>
       </c>
       <c r="K2" s="15" t="s">
         <v>8</v>
       </c>
       <c r="L2" s="1"/>
-      <c r="M2" s="13" t="s">
+      <c r="M2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="N2" s="13" t="s">
+      <c r="N2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="13"/>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="13"/>
-      <c r="S2" s="13"/>
-      <c r="T2" s="13" t="s">
+      <c r="O2" s="14"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="14"/>
+      <c r="S2" s="14"/>
+      <c r="T2" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="U2" s="13" t="s">
+      <c r="U2" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="V2" s="14" t="s">
+      <c r="V2" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="W2" s="14" t="s">
+      <c r="W2" s="16" t="s">
         <v>13</v>
       </c>
       <c r="X2" s="2" t="s">
@@ -702,18 +702,18 @@
       </c>
     </row>
     <row r="3" spans="2:28" ht="45">
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
       <c r="I3" s="15"/>
-      <c r="J3" s="13"/>
+      <c r="J3" s="14"/>
       <c r="K3" s="15"/>
       <c r="L3" s="1"/>
-      <c r="M3" s="13"/>
+      <c r="M3" s="14"/>
       <c r="N3" s="1" t="s">
         <v>15</v>
       </c>
@@ -732,10 +732,10 @@
       <c r="S3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
-      <c r="V3" s="14"/>
-      <c r="W3" s="14"/>
+      <c r="T3" s="14"/>
+      <c r="U3" s="14"/>
+      <c r="V3" s="16"/>
+      <c r="W3" s="16"/>
       <c r="X3" s="2"/>
     </row>
     <row r="4" spans="2:28">
@@ -756,13 +756,13 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I4" s="4">
         <v>25</v>
       </c>
       <c r="J4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K4" s="4">
         <v>3</v>
@@ -793,13 +793,13 @@
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I5" s="4">
         <v>4</v>
       </c>
       <c r="J5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K5" s="4">
         <v>12</v>
@@ -830,13 +830,13 @@
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I6" s="4">
         <v>1260</v>
       </c>
       <c r="J6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K6" s="4">
         <v>12</v>
@@ -869,13 +869,13 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I7" s="4">
         <v>86</v>
       </c>
       <c r="J7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K7" s="4">
         <v>3</v>
@@ -906,13 +906,13 @@
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I8" s="4">
         <v>10</v>
       </c>
       <c r="J8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>36</v>
@@ -941,13 +941,13 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I9" s="4">
         <v>1277</v>
       </c>
       <c r="J9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K9" s="4"/>
       <c r="N9" s="8" t="s">
@@ -981,7 +981,7 @@
     </row>
     <row r="10" spans="2:28">
       <c r="B10" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="11">
@@ -1015,7 +1015,7 @@
     </row>
     <row r="11" spans="2:28">
       <c r="B11" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="11">
@@ -1049,7 +1049,7 @@
     </row>
     <row r="12" spans="2:28">
       <c r="B12" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C12" s="11"/>
       <c r="D12" s="11">
@@ -1083,7 +1083,7 @@
     </row>
     <row r="13" spans="2:28">
       <c r="B13" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="11">
@@ -1117,7 +1117,7 @@
     </row>
     <row r="14" spans="2:28">
       <c r="B14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D14">
         <v>15</v>
@@ -1133,13 +1133,13 @@
         <v>1</v>
       </c>
       <c r="H14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I14" s="4">
         <v>10</v>
       </c>
       <c r="J14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K14" s="4">
         <v>12</v>
@@ -1151,7 +1151,7 @@
         <v>2</v>
       </c>
       <c r="N14" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O14" s="9">
         <v>5</v>
@@ -1178,7 +1178,7 @@
     </row>
     <row r="15" spans="2:28">
       <c r="B15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D15">
         <v>16</v>
@@ -1194,25 +1194,25 @@
         <v>1</v>
       </c>
       <c r="H15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I15" s="4">
         <v>10</v>
       </c>
       <c r="J15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K15" s="4">
         <v>3</v>
       </c>
       <c r="L15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M15" s="4">
         <v>6</v>
       </c>
       <c r="N15" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O15" s="9">
         <v>1</v>
@@ -1352,7 +1352,7 @@
         <v>0x16</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="G19" s="11"/>
       <c r="H19" s="11"/>
@@ -1375,7 +1375,7 @@
     </row>
     <row r="20" spans="2:24">
       <c r="B20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D20">
         <v>23</v>
@@ -1385,19 +1385,19 @@
         <v>0x17</v>
       </c>
       <c r="F20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G20">
         <v>1</v>
       </c>
       <c r="H20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I20" s="4">
         <v>0</v>
       </c>
       <c r="J20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K20" s="4">
         <v>2</v>
@@ -1409,7 +1409,7 @@
         <v>4</v>
       </c>
       <c r="N20" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="O20" s="9">
         <v>0</v>
@@ -1433,7 +1433,7 @@
         <v>2</v>
       </c>
       <c r="V20" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="W20" s="5">
         <v>63</v>
@@ -1453,7 +1453,7 @@
         <v>0x18</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G21" s="11"/>
       <c r="H21" s="11"/>
@@ -1469,10 +1469,10 @@
       <c r="R21" s="11"/>
       <c r="S21" s="11"/>
       <c r="T21" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="U21" s="12" t="s">
         <v>68</v>
-      </c>
-      <c r="U21" s="12" t="s">
-        <v>69</v>
       </c>
       <c r="V21" s="5"/>
       <c r="W21" s="5"/>
@@ -1480,21 +1480,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="N2:S2"/>
+    <mergeCell ref="T2:T3"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="M2:M3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:E3"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:S2"/>
-    <mergeCell ref="T2:T3"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="W2:W3"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
actualizacion de libreria rust, ahora incluye mas metricas estadisiticas para RegisterUnits, se observa que el tiempo de benchmark se reredujo, previamente era de 15 veces ahora se acerca a 5 veces, tambien se implemento jupyter notebook en el repositorio para realizar pruebas sin tener que usar la pynq en mano, tambien en este momento las tests se encuentran desactualizadas, no funcionaran, y fallaran, se actualizo el README, se agrego un requirements.txt para pip y python con el ambiente virtual, se agregaron las traces de una lectura hecha por el intermediador de la PYNQ en jupyter/data/input/
</commit_message>
<xml_diff>
--- a/modbus.xlsx
+++ b/modbus.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\windows\projects\rust\firerust\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF1632D5-EEB3-49F5-BCEC-6E85FABDB37C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A135E1B-2076-465A-B8DC-363062CFA6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="initial_process" sheetId="1" r:id="rId1"/>
+    <sheet name="rolling_window" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="76">
   <si>
     <t>MODBUS INSTRUCTION SAMPLE</t>
   </si>
@@ -270,6 +271,12 @@
   </si>
   <si>
     <t>mask_write_register</t>
+  </si>
+  <si>
+    <t>average value reg</t>
+  </si>
+  <si>
+    <t>quartile 1</t>
   </si>
 </sst>
 </file>
@@ -374,16 +381,16 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -620,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:AB21"/>
+  <dimension ref="B2:AD21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="45.5703125" customWidth="1"/>
@@ -636,84 +643,86 @@
     <col min="13" max="13" width="7.5703125" customWidth="1"/>
     <col min="14" max="14" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="9" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.5703125" customWidth="1"/>
-    <col min="17" max="17" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.28515625" customWidth="1"/>
-    <col min="19" max="19" width="8" customWidth="1"/>
-    <col min="20" max="22" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="9.5703125" customWidth="1"/>
+    <col min="18" max="18" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="8.28515625" customWidth="1"/>
+    <col min="21" max="21" width="8" customWidth="1"/>
+    <col min="22" max="24" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="38.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:28" ht="30" customHeight="1">
-      <c r="B2" s="13" t="s">
+    <row r="2" spans="2:30" ht="30" customHeight="1">
+      <c r="B2" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="13"/>
-      <c r="F2" s="14" t="s">
+      <c r="E2" s="16"/>
+      <c r="F2" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="H2" s="13" t="s">
         <v>5</v>
       </c>
       <c r="I2" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="13" t="s">
         <v>7</v>
       </c>
       <c r="K2" s="15" t="s">
         <v>8</v>
       </c>
       <c r="L2" s="1"/>
-      <c r="M2" s="14" t="s">
+      <c r="M2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="14"/>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
-      <c r="R2" s="14"/>
-      <c r="S2" s="14"/>
-      <c r="T2" s="14" t="s">
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13"/>
+      <c r="T2" s="13"/>
+      <c r="U2" s="13"/>
+      <c r="V2" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="U2" s="14" t="s">
+      <c r="W2" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="V2" s="16" t="s">
+      <c r="X2" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="W2" s="16" t="s">
+      <c r="Y2" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="X2" s="2" t="s">
+      <c r="Z2" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:28" ht="45">
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
+    <row r="3" spans="2:30" ht="45">
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
       <c r="I3" s="15"/>
-      <c r="J3" s="14"/>
+      <c r="J3" s="13"/>
       <c r="K3" s="15"/>
       <c r="L3" s="1"/>
-      <c r="M3" s="14"/>
+      <c r="M3" s="13"/>
       <c r="N3" s="1" t="s">
         <v>15</v>
       </c>
@@ -724,21 +733,27 @@
         <v>17</v>
       </c>
       <c r="Q3" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="R3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="S3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="S3" s="1" t="s">
+      <c r="T3" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="U3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
-      <c r="V3" s="16"/>
-      <c r="W3" s="16"/>
-      <c r="X3" s="2"/>
-    </row>
-    <row r="4" spans="2:28">
+      <c r="V3" s="13"/>
+      <c r="W3" s="13"/>
+      <c r="X3" s="14"/>
+      <c r="Y3" s="14"/>
+      <c r="Z3" s="2"/>
+    </row>
+    <row r="4" spans="2:30">
       <c r="B4" t="s">
         <v>21</v>
       </c>
@@ -767,15 +782,15 @@
       <c r="K4" s="4">
         <v>3</v>
       </c>
-      <c r="V4" s="5" t="s">
+      <c r="X4" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="W4" s="5" t="s">
+      <c r="Y4" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="X4" s="6"/>
-    </row>
-    <row r="5" spans="2:28">
+      <c r="Z4" s="6"/>
+    </row>
+    <row r="5" spans="2:30">
       <c r="B5" t="s">
         <v>25</v>
       </c>
@@ -804,15 +819,15 @@
       <c r="K5" s="4">
         <v>12</v>
       </c>
-      <c r="V5" s="5">
+      <c r="X5" s="5">
         <v>39</v>
       </c>
-      <c r="W5" s="5" t="s">
+      <c r="Y5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="X5" s="6"/>
-    </row>
-    <row r="6" spans="2:28">
+      <c r="Z5" s="6"/>
+    </row>
+    <row r="6" spans="2:30">
       <c r="B6" t="s">
         <v>28</v>
       </c>
@@ -841,17 +856,17 @@
       <c r="K6" s="4">
         <v>12</v>
       </c>
-      <c r="V6" s="5">
+      <c r="X6" s="5">
         <v>85</v>
       </c>
-      <c r="W6" s="5" t="s">
+      <c r="Y6" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="X6" s="6"/>
-      <c r="AA6" s="7"/>
-      <c r="AB6" s="7"/>
-    </row>
-    <row r="7" spans="2:28">
+      <c r="Z6" s="6"/>
+      <c r="AC6" s="7"/>
+      <c r="AD6" s="7"/>
+    </row>
+    <row r="7" spans="2:30">
       <c r="B7" t="s">
         <v>31</v>
       </c>
@@ -880,15 +895,15 @@
       <c r="K7" s="4">
         <v>3</v>
       </c>
-      <c r="V7" s="5">
+      <c r="X7" s="5">
         <v>50</v>
       </c>
-      <c r="W7" s="5" t="s">
+      <c r="Y7" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="X7" s="6"/>
-    </row>
-    <row r="8" spans="2:28">
+      <c r="Z7" s="6"/>
+    </row>
+    <row r="8" spans="2:30">
       <c r="B8" t="s">
         <v>34</v>
       </c>
@@ -917,13 +932,13 @@
       <c r="K8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="V8" s="5"/>
-      <c r="W8" s="5"/>
-      <c r="X8" s="6" t="s">
+      <c r="X8" s="5"/>
+      <c r="Y8" s="5"/>
+      <c r="Z8" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="2:28">
+    <row r="9" spans="2:30">
       <c r="B9" t="s">
         <v>38</v>
       </c>
@@ -959,27 +974,29 @@
       <c r="P9" s="9">
         <v>1757</v>
       </c>
-      <c r="Q9" s="9">
+      <c r="Q9" s="9"/>
+      <c r="R9" s="9">
         <f>MEDIAN(O9:P9)</f>
         <v>1757</v>
       </c>
-      <c r="R9" s="9">
+      <c r="S9" s="9">
         <v>1757</v>
       </c>
-      <c r="S9" s="9">
+      <c r="T9" s="9"/>
+      <c r="U9" s="9">
         <v>4</v>
       </c>
-      <c r="T9" s="8"/>
-      <c r="U9" s="8"/>
-      <c r="V9" s="5" t="s">
+      <c r="V9" s="8"/>
+      <c r="W9" s="8"/>
+      <c r="X9" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="W9" s="5" t="s">
+      <c r="Y9" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="X9" s="6"/>
-    </row>
-    <row r="10" spans="2:28">
+      <c r="Z9" s="6"/>
+    </row>
+    <row r="10" spans="2:30">
       <c r="B10" s="10" t="s">
         <v>70</v>
       </c>
@@ -1009,11 +1026,13 @@
       <c r="S10" s="11"/>
       <c r="T10" s="11"/>
       <c r="U10" s="11"/>
-      <c r="V10" s="5"/>
-      <c r="W10" s="5"/>
-      <c r="X10" s="6"/>
-    </row>
-    <row r="11" spans="2:28">
+      <c r="V10" s="11"/>
+      <c r="W10" s="11"/>
+      <c r="X10" s="5"/>
+      <c r="Y10" s="5"/>
+      <c r="Z10" s="6"/>
+    </row>
+    <row r="11" spans="2:30">
       <c r="B11" s="11" t="s">
         <v>69</v>
       </c>
@@ -1043,11 +1062,13 @@
       <c r="S11" s="11"/>
       <c r="T11" s="11"/>
       <c r="U11" s="11"/>
-      <c r="V11" s="5"/>
-      <c r="W11" s="5"/>
-      <c r="X11" s="6"/>
-    </row>
-    <row r="12" spans="2:28">
+      <c r="V11" s="11"/>
+      <c r="W11" s="11"/>
+      <c r="X11" s="5"/>
+      <c r="Y11" s="5"/>
+      <c r="Z11" s="6"/>
+    </row>
+    <row r="12" spans="2:30">
       <c r="B12" s="11" t="s">
         <v>71</v>
       </c>
@@ -1077,11 +1098,13 @@
       <c r="S12" s="11"/>
       <c r="T12" s="11"/>
       <c r="U12" s="11"/>
-      <c r="V12" s="5"/>
-      <c r="W12" s="5"/>
-      <c r="X12" s="6"/>
-    </row>
-    <row r="13" spans="2:28">
+      <c r="V12" s="11"/>
+      <c r="W12" s="11"/>
+      <c r="X12" s="5"/>
+      <c r="Y12" s="5"/>
+      <c r="Z12" s="6"/>
+    </row>
+    <row r="13" spans="2:30">
       <c r="B13" s="10" t="s">
         <v>72</v>
       </c>
@@ -1111,11 +1134,13 @@
       <c r="S13" s="11"/>
       <c r="T13" s="11"/>
       <c r="U13" s="11"/>
-      <c r="V13" s="5"/>
-      <c r="W13" s="5"/>
-      <c r="X13" s="6"/>
-    </row>
-    <row r="14" spans="2:28">
+      <c r="V13" s="11"/>
+      <c r="W13" s="11"/>
+      <c r="X13" s="5"/>
+      <c r="Y13" s="5"/>
+      <c r="Z13" s="6"/>
+    </row>
+    <row r="14" spans="2:30">
       <c r="B14" t="s">
         <v>65</v>
       </c>
@@ -1159,24 +1184,26 @@
       <c r="P14" s="9">
         <v>5</v>
       </c>
-      <c r="Q14" s="9">
-        <v>5</v>
-      </c>
+      <c r="Q14" s="9"/>
       <c r="R14" s="9">
         <v>5</v>
       </c>
       <c r="S14" s="9">
+        <v>5</v>
+      </c>
+      <c r="T14" s="9"/>
+      <c r="U14" s="9">
         <v>14</v>
       </c>
-      <c r="V14" s="5" t="s">
+      <c r="X14" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="W14" s="5">
+      <c r="Y14" s="5">
         <v>95</v>
       </c>
-      <c r="X14" s="6"/>
-    </row>
-    <row r="15" spans="2:28">
+      <c r="Z14" s="6"/>
+    </row>
+    <row r="15" spans="2:30">
       <c r="B15" t="s">
         <v>62</v>
       </c>
@@ -1220,24 +1247,26 @@
       <c r="P15" s="9">
         <v>4</v>
       </c>
-      <c r="Q15" s="9">
+      <c r="Q15" s="9"/>
+      <c r="R15" s="9">
         <v>2.5</v>
       </c>
-      <c r="R15" s="9">
+      <c r="S15" s="9">
         <v>10</v>
       </c>
-      <c r="S15" s="9">
+      <c r="T15" s="9"/>
+      <c r="U15" s="9">
         <v>27</v>
       </c>
-      <c r="V15" s="5" t="s">
+      <c r="X15" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="W15" s="5" t="s">
+      <c r="Y15" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="X15" s="6"/>
-    </row>
-    <row r="16" spans="2:28">
+      <c r="Z15" s="6"/>
+    </row>
+    <row r="16" spans="2:30">
       <c r="B16" s="10" t="s">
         <v>43</v>
       </c>
@@ -1267,11 +1296,13 @@
       <c r="S16" s="11"/>
       <c r="T16" s="11"/>
       <c r="U16" s="11"/>
-      <c r="V16" s="5"/>
-      <c r="W16" s="5"/>
-      <c r="X16" s="6"/>
-    </row>
-    <row r="17" spans="2:24">
+      <c r="V16" s="11"/>
+      <c r="W16" s="11"/>
+      <c r="X16" s="5"/>
+      <c r="Y16" s="5"/>
+      <c r="Z16" s="6"/>
+    </row>
+    <row r="17" spans="2:26">
       <c r="B17" s="11" t="s">
         <v>43</v>
       </c>
@@ -1301,11 +1332,13 @@
       <c r="S17" s="11"/>
       <c r="T17" s="11"/>
       <c r="U17" s="11"/>
-      <c r="V17" s="5"/>
-      <c r="W17" s="5"/>
-      <c r="X17" s="6"/>
-    </row>
-    <row r="18" spans="2:24">
+      <c r="V17" s="11"/>
+      <c r="W17" s="11"/>
+      <c r="X17" s="5"/>
+      <c r="Y17" s="5"/>
+      <c r="Z17" s="6"/>
+    </row>
+    <row r="18" spans="2:26">
       <c r="B18" s="11" t="s">
         <v>43</v>
       </c>
@@ -1335,11 +1368,13 @@
       <c r="S18" s="11"/>
       <c r="T18" s="11"/>
       <c r="U18" s="11"/>
-      <c r="V18" s="5"/>
-      <c r="W18" s="5"/>
-      <c r="X18" s="6"/>
-    </row>
-    <row r="19" spans="2:24">
+      <c r="V18" s="11"/>
+      <c r="W18" s="11"/>
+      <c r="X18" s="5"/>
+      <c r="Y18" s="5"/>
+      <c r="Z18" s="6"/>
+    </row>
+    <row r="19" spans="2:26">
       <c r="B19" s="10" t="s">
         <v>43</v>
       </c>
@@ -1369,11 +1404,13 @@
       <c r="S19" s="11"/>
       <c r="T19" s="11"/>
       <c r="U19" s="11"/>
-      <c r="V19" s="5"/>
-      <c r="W19" s="5"/>
-      <c r="X19" s="6"/>
-    </row>
-    <row r="20" spans="2:24">
+      <c r="V19" s="11"/>
+      <c r="W19" s="11"/>
+      <c r="X19" s="5"/>
+      <c r="Y19" s="5"/>
+      <c r="Z19" s="6"/>
+    </row>
+    <row r="20" spans="2:26">
       <c r="B20" t="s">
         <v>55</v>
       </c>
@@ -1417,30 +1454,32 @@
       <c r="P20" s="9">
         <v>2</v>
       </c>
-      <c r="Q20" s="9">
+      <c r="Q20" s="9"/>
+      <c r="R20" s="9">
         <v>0.75</v>
       </c>
-      <c r="R20" s="9">
+      <c r="S20" s="9">
         <v>3</v>
       </c>
-      <c r="S20" s="9">
+      <c r="T20" s="9"/>
+      <c r="U20" s="9">
         <v>30</v>
       </c>
-      <c r="T20" s="4">
+      <c r="V20" s="4">
         <v>10</v>
       </c>
-      <c r="U20" s="4">
+      <c r="W20" s="4">
         <v>2</v>
       </c>
-      <c r="V20" s="5" t="s">
+      <c r="X20" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="W20" s="5">
+      <c r="Y20" s="5">
         <v>63</v>
       </c>
-      <c r="X20" s="6"/>
-    </row>
-    <row r="21" spans="2:24">
+      <c r="Z20" s="6"/>
+    </row>
+    <row r="21" spans="2:26">
       <c r="B21" s="10" t="s">
         <v>43</v>
       </c>
@@ -1468,36 +1507,47 @@
       <c r="Q21" s="11"/>
       <c r="R21" s="11"/>
       <c r="S21" s="11"/>
-      <c r="T21" s="12" t="s">
+      <c r="T21" s="11"/>
+      <c r="U21" s="11"/>
+      <c r="V21" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="U21" s="12" t="s">
+      <c r="W21" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="V21" s="5"/>
-      <c r="W21" s="5"/>
-      <c r="X21" s="6"/>
+      <c r="X21" s="5"/>
+      <c r="Y21" s="5"/>
+      <c r="Z21" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="N2:S2"/>
-    <mergeCell ref="T2:T3"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
     <mergeCell ref="M2:M3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:E3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="N2:U2"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="X2:X3"/>
+    <mergeCell ref="Y2:Y3"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA986AEA-5F27-4EB2-9BF2-70A0646B7917}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>